<commit_message>
Record corrected screenshot outreach delivery
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC9DC5C-59CC-481B-A985-C6F19469CD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8E84F1-A3E9-430B-8301-D44BE589C554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -185,9 +185,6 @@
     <t>Hello Mrs. Wilson's Cafe team. I prepared a simple website preview for your cafe using public business details. I can customize it, deploy it, and add backend features if you are interested, with a small budget agreed in advance. May I share the preview?</t>
   </si>
   <si>
-    <t>2 screenshots + GitHub website link</t>
-  </si>
-  <si>
     <t>Draft only</t>
   </si>
   <si>
@@ -215,10 +212,13 @@
     <t>Owner review; confirm facts, price, approval, then deploy</t>
   </si>
   <si>
-    <t>Sent - Delivered 2026-10-20 3:34 pm</t>
-  </si>
-  <si>
-    <t>Sent and Delivered</t>
+    <t>Resent - Delivered 2026-10-20 3:37 pm</t>
+  </si>
+  <si>
+    <t>Public raw image links: raw.githubusercontent.com home + services</t>
+  </si>
+  <si>
+    <t>Corrected and Delivered</t>
   </si>
 </sst>
 </file>
@@ -624,10 +624,10 @@
         <v>6</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="120" x14ac:dyDescent="0.25">
@@ -638,22 +638,22 @@
         <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -702,7 +702,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>30</v>
@@ -711,7 +711,7 @@
         <v>47</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
@@ -722,13 +722,13 @@
         <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Record Bune delivery work in tracker
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8E84F1-A3E9-430B-8301-D44BE589C554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA292A3E-61FE-4CB3-8060-FBE2FF7E2905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -219,6 +219,33 @@
   </si>
   <si>
     <t>Corrected and Delivered</t>
+  </si>
+  <si>
+    <t>Bune - The Coffee Room</t>
+  </si>
+  <si>
+    <t>Prepared - pending send</t>
+  </si>
+  <si>
+    <t>+91 3346014070</t>
+  </si>
+  <si>
+    <t>Website preview message with template attribution and MultiMax footer</t>
+  </si>
+  <si>
+    <t>2 public raw screenshot links</t>
+  </si>
+  <si>
+    <t>sites/bune-the-coffee-room/index.html</t>
+  </si>
+  <si>
+    <t>Uploaded commit eab021b</t>
+  </si>
+  <si>
+    <t>Prepared; pending delivery</t>
+  </si>
+  <si>
+    <t>Owner review; confirm template license, facts, price, approval, then deploy</t>
   </si>
 </sst>
 </file>
@@ -268,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -280,6 +307,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -594,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C11FA4A-69D6-4815-95B1-E4309A30900A}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -656,6 +686,32 @@
         <v>56</v>
       </c>
     </row>
+    <row r="3" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -663,7 +719,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AE1D06A-CF40-4DAF-AA1C-618059D935F9}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -714,7 +770,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -732,6 +788,26 @@
       </c>
       <c r="F3" s="1" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Bune WhatsApp channel unavailable
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA292A3E-61FE-4CB3-8060-FBE2FF7E2905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B76425-8C96-469B-B53B-552C40FD9053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -224,15 +224,9 @@
     <t>Bune - The Coffee Room</t>
   </si>
   <si>
-    <t>Prepared - pending send</t>
-  </si>
-  <si>
     <t>+91 3346014070</t>
   </si>
   <si>
-    <t>Website preview message with template attribution and MultiMax footer</t>
-  </si>
-  <si>
     <t>2 public raw screenshot links</t>
   </si>
   <si>
@@ -242,10 +236,16 @@
     <t>Uploaded commit eab021b</t>
   </si>
   <si>
-    <t>Prepared; pending delivery</t>
-  </si>
-  <si>
     <t>Owner review; confirm template license, facts, price, approval, then deploy</t>
+  </si>
+  <si>
+    <t>Not sent - number not registered on WhatsApp</t>
+  </si>
+  <si>
+    <t>Checked 2026-10-20</t>
+  </si>
+  <si>
+    <t>Not sent - number not on WhatsApp</t>
   </si>
 </sst>
 </file>
@@ -691,16 +691,16 @@
         <v>60</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>48</v>
@@ -709,7 +709,7 @@
         <v>55</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -790,7 +790,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -798,16 +798,16 @@
         <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add verified Bune contact fallback rule
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B76425-8C96-469B-B53B-552C40FD9053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714FCD26-AF95-427E-BCF1-7D20EEC85211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="68">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -224,9 +224,6 @@
     <t>Bune - The Coffee Room</t>
   </si>
   <si>
-    <t>+91 3346014070</t>
-  </si>
-  <si>
     <t>2 public raw screenshot links</t>
   </si>
   <si>
@@ -236,16 +233,16 @@
     <t>Uploaded commit eab021b</t>
   </si>
   <si>
-    <t>Owner review; confirm template license, facts, price, approval, then deploy</t>
-  </si>
-  <si>
-    <t>Not sent - number not registered on WhatsApp</t>
-  </si>
-  <si>
-    <t>Checked 2026-10-20</t>
-  </si>
-  <si>
-    <t>Not sent - number not on WhatsApp</t>
+    <t>Pending WhatsApp check</t>
+  </si>
+  <si>
+    <t>+91 9330321589</t>
+  </si>
+  <si>
+    <t>Found in second public listing search; check before sending</t>
+  </si>
+  <si>
+    <t>Check verified number; if no channel is found, ask owner in WhatsApp</t>
   </si>
 </sst>
 </file>
@@ -691,16 +688,16 @@
         <v>60</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>48</v>
@@ -709,7 +706,7 @@
         <v>55</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -798,16 +795,16 @@
         <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Bune contact channel unavailable
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714FCD26-AF95-427E-BCF1-7D20EEC85211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CC783C-0904-435C-849B-7B8388960018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -233,16 +233,19 @@
     <t>Uploaded commit eab021b</t>
   </si>
   <si>
-    <t>Pending WhatsApp check</t>
-  </si>
-  <si>
     <t>+91 9330321589</t>
   </si>
   <si>
-    <t>Found in second public listing search; check before sending</t>
-  </si>
-  <si>
-    <t>Check verified number; if no channel is found, ask owner in WhatsApp</t>
+    <t>Not sent - number not registered on WhatsApp</t>
+  </si>
+  <si>
+    <t>Checked through connected WhatsApp Web 2026-10-20; owner contact required</t>
+  </si>
+  <si>
+    <t>Not sent - number not on WhatsApp</t>
+  </si>
+  <si>
+    <t>Ask owner in WhatsApp for a verified contact channel</t>
   </si>
 </sst>
 </file>
@@ -683,7 +686,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>60</v>
       </c>
@@ -697,7 +700,7 @@
         <v>63</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>48</v>
@@ -706,7 +709,7 @@
         <v>55</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -787,7 +790,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -795,10 +798,10 @@
         <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Add same-niche contact fallback workflow
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CC783C-0904-435C-849B-7B8388960018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3A027D-AC1D-436B-8071-1BE07798C54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
   <sheets>
-    <sheet name="Delivery" sheetId="3" r:id="rId1"/>
-    <sheet name="Messages" sheetId="2" r:id="rId2"/>
-    <sheet name="Work" sheetId="1" r:id="rId3"/>
+    <sheet name="Workflow Rules" sheetId="4" r:id="rId1"/>
+    <sheet name="Delivery" sheetId="3" r:id="rId2"/>
+    <sheet name="Messages" sheetId="2" r:id="rId3"/>
+    <sheet name="Work" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="80">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -246,13 +247,46 @@
   </si>
   <si>
     <t>Ask owner in WhatsApp for a verified contact channel</t>
+  </si>
+  <si>
+    <t>Rule</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>No usable WhatsApp contact</t>
+  </si>
+  <si>
+    <t>Record the reason, ask the owner for a verified contact channel in WhatsApp when needed, and do not claim outreach was sent.</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Same-niche fallback</t>
+  </si>
+  <si>
+    <t>Continue with another same-niche local business that has no official website and a usable public contact channel.</t>
+  </si>
+  <si>
+    <t>No contactable prospect</t>
+  </si>
+  <si>
+    <t>Record owner_contact_required and wait for a verified channel or new prospect; do not stop the overall workflow permanently.</t>
+  </si>
+  <si>
+    <t>Website footer</t>
+  </si>
+  <si>
+    <t>Every generated website must show Developed by MultiMax.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -264,6 +298,14 @@
       <b/>
       <sz val="11"/>
       <color indexed="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -295,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -310,6 +352,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,6 +666,76 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E0CBB4-9F75-4C43-B3FF-DF4CD3FDFD21}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="117.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C11FA4A-69D6-4815-95B1-E4309A30900A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -717,7 +830,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AE1D06A-CF40-4DAF-AA1C-618059D935F9}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -815,7 +928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEAD64A3-3D57-402D-8DCE-986984D1D9A0}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Record Lighthouse Cafe 10 AM test
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3A027D-AC1D-436B-8071-1BE07798C54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEA5545-7330-46E3-9F5E-2EEEC53AE014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="90">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -280,6 +280,36 @@
   </si>
   <si>
     <t>Every generated website must show Developed by MultiMax.</t>
+  </si>
+  <si>
+    <t>The Lighthouse Cafe</t>
+  </si>
+  <si>
+    <t>Draft prepared - pending WhatsApp check</t>
+  </si>
+  <si>
+    <t>+91 8910780424</t>
+  </si>
+  <si>
+    <t>Website preview prepared by qwen3:4b</t>
+  </si>
+  <si>
+    <t>GitHub site link; screenshots pending capture</t>
+  </si>
+  <si>
+    <t>sites/the-lighthouse-cafe/index.html</t>
+  </si>
+  <si>
+    <t>Pending screenshot capture</t>
+  </si>
+  <si>
+    <t>Pushed by Ollama run</t>
+  </si>
+  <si>
+    <t>Pending WhatsApp check</t>
+  </si>
+  <si>
+    <t>Owner review; verify contact, facts, price, approval, then deploy</t>
   </si>
 </sst>
 </file>
@@ -737,7 +767,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C11FA4A-69D6-4815-95B1-E4309A30900A}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -825,6 +855,32 @@
         <v>68</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" t="s">
+        <v>89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -832,7 +888,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AE1D06A-CF40-4DAF-AA1C-618059D935F9}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -921,6 +977,26 @@
       </c>
       <c r="F4" s="5" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace Lighthouse site with ThemeWagon Tasty template
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEA5545-7330-46E3-9F5E-2EEEC53AE014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686DDF79-1E50-4BFD-9AB7-B53FDE19F2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -294,15 +294,9 @@
     <t>Website preview prepared by qwen3:4b</t>
   </si>
   <si>
-    <t>GitHub site link; screenshots pending capture</t>
-  </si>
-  <si>
     <t>sites/the-lighthouse-cafe/index.html</t>
   </si>
   <si>
-    <t>Pending screenshot capture</t>
-  </si>
-  <si>
     <t>Pushed by Ollama run</t>
   </si>
   <si>
@@ -310,6 +304,12 @@
   </si>
   <si>
     <t>Owner review; verify contact, facts, price, approval, then deploy</t>
+  </si>
+  <si>
+    <t>Public raw homepage screenshot link</t>
+  </si>
+  <si>
+    <t>1 file in work/screenshots/</t>
   </si>
 </sst>
 </file>
@@ -860,16 +860,16 @@
         <v>80</v>
       </c>
       <c r="B4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" t="s">
         <v>85</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>86</v>
-      </c>
-      <c r="D4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" t="s">
-        <v>88</v>
       </c>
       <c r="F4" t="s">
         <v>48</v>
@@ -878,7 +878,7 @@
         <v>55</v>
       </c>
       <c r="H4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -996,7 +996,7 @@
         <v>83</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean template footer and record Lighthouse outreach
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686DDF79-1E50-4BFD-9AB7-B53FDE19F2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8BF404-F38E-4DCC-B711-17D7B8132726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="89">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -285,31 +285,28 @@
     <t>The Lighthouse Cafe</t>
   </si>
   <si>
-    <t>Draft prepared - pending WhatsApp check</t>
-  </si>
-  <si>
     <t>+91 8910780424</t>
   </si>
   <si>
-    <t>Website preview prepared by qwen3:4b</t>
-  </si>
-  <si>
     <t>sites/the-lighthouse-cafe/index.html</t>
   </si>
   <si>
     <t>Pushed by Ollama run</t>
   </si>
   <si>
-    <t>Pending WhatsApp check</t>
-  </si>
-  <si>
-    <t>Owner review; verify contact, facts, price, approval, then deploy</t>
-  </si>
-  <si>
     <t>Public raw homepage screenshot link</t>
   </si>
   <si>
     <t>1 file in work/screenshots/</t>
+  </si>
+  <si>
+    <t>Sent - Delivered 2026-10-20 7:16 pm</t>
+  </si>
+  <si>
+    <t>Corrected ThemeWagon-based preview sent</t>
+  </si>
+  <si>
+    <t>Sent - Delivered</t>
   </si>
 </sst>
 </file>
@@ -860,16 +857,16 @@
         <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
         <v>48</v>
@@ -878,7 +875,7 @@
         <v>55</v>
       </c>
       <c r="H4" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -987,16 +984,16 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" t="s">
         <v>81</v>
       </c>
-      <c r="D5" t="s">
-        <v>82</v>
-      </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add MultiMax outreach follow-up
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8BF404-F38E-4DCC-B711-17D7B8132726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA7280D-D500-41C5-AFA1-7F01200EC992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -300,13 +300,13 @@
     <t>1 file in work/screenshots/</t>
   </si>
   <si>
-    <t>Sent - Delivered 2026-10-20 7:16 pm</t>
-  </si>
-  <si>
-    <t>Corrected ThemeWagon-based preview sent</t>
-  </si>
-  <si>
     <t>Sent - Delivered</t>
+  </si>
+  <si>
+    <t>Sent - Delivered 2026-10-20 7:16 pm; follow-up delivered 7:22 pm</t>
+  </si>
+  <si>
+    <t>Preview + MultiMax company details + follow-up CTA sent</t>
   </si>
 </sst>
 </file>
@@ -866,7 +866,7 @@
         <v>83</v>
       </c>
       <c r="E4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F4" t="s">
         <v>48</v>
@@ -984,13 +984,13 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D5" t="s">
         <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F5" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
Standardize Amala MultiMax outreach introduction
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA7280D-D500-41C5-AFA1-7F01200EC992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759C83D3-0277-4EC7-A2E0-0C9A47F25D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -303,10 +303,10 @@
     <t>Sent - Delivered</t>
   </si>
   <si>
-    <t>Sent - Delivered 2026-10-20 7:16 pm; follow-up delivered 7:22 pm</t>
-  </si>
-  <si>
-    <t>Preview + MultiMax company details + follow-up CTA sent</t>
+    <t>Sent - Delivered 7:16 pm; follow-up 7:22 pm; intro 7:24 pm</t>
+  </si>
+  <si>
+    <t>Amala + MultiMax intro, preview CTA and low-budget offer delivered</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add standard outreach rule for every 10 AM run
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759C83D3-0277-4EC7-A2E0-0C9A47F25D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CD48A9-AC2E-4148-83DB-249F236DE51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -307,6 +307,15 @@
   </si>
   <si>
     <t>Amala + MultiMax intro, preview CTA and low-budget offer delivered</t>
+  </si>
+  <si>
+    <t>Standard Amala/MultiMax outreach</t>
+  </si>
+  <si>
+    <t>Use the exact Amala introduction, explain MultiMax affordable local-business websites, mention no dedicated website, offer a low agreed budget, and ask the owner to reply for the preview/full details.</t>
+  </si>
+  <si>
+    <t>Active for every 10 AM run</t>
   </si>
 </sst>
 </file>
@@ -694,12 +703,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E0CBB4-9F75-4C43-B3FF-DF4CD3FDFD21}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="117.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="185.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -755,6 +764,17 @@
       </c>
       <c r="C5" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Authorize automatic outreach for 10 AM workflow
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CD48A9-AC2E-4148-83DB-249F236DE51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D580ED83-AA46-454A-BE09-B48672F0157F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="94">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -316,6 +316,12 @@
   </si>
   <si>
     <t>Active for every 10 AM run</t>
+  </si>
+  <si>
+    <t>No per-run permission</t>
+  </si>
+  <si>
+    <t>Qwen completes the 10 AM build, updates GitHub/Excel, and sends through the connected WhatsApp/email adapter automatically; report the exact result afterward.</t>
   </si>
 </sst>
 </file>
@@ -703,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E0CBB4-9F75-4C43-B3FF-DF4CD3FDFD21}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -774,6 +780,17 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand 10 AM discovery worldwide
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SARANYA\.codex\visualizations\2026\10\20\01a15877-7be2-7170-a677-48cdbe8236c5\10-am-office-work\work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D580ED83-AA46-454A-BE09-B48672F0157F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82880012-B64A-4FD5-A508-1A94B36B2FC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{644FE1C5-50C8-4BF1-AE1F-F48396027018}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="96">
   <si>
     <t>10 AM Office Work</t>
   </si>
@@ -322,6 +322,12 @@
   </si>
   <si>
     <t>Qwen completes the 10 AM build, updates GitHub/Excel, and sends through the connected WhatsApp/email adapter automatically; report the exact result afterward.</t>
+  </si>
+  <si>
+    <t>Worldwide discovery</t>
+  </si>
+  <si>
+    <t>Search businesses globally. If the local queue is empty or a contact channel fails, find another same-niche no-website prospect in another city or country before reporting no work.</t>
   </si>
 </sst>
 </file>
@@ -709,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E0CBB4-9F75-4C43-B3FF-DF4CD3FDFD21}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -791,6 +797,17 @@
         <v>93</v>
       </c>
       <c r="C7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Record No. 41 Coffee WhatsApp result
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -822,7 +822,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Queued for connected adapter</t>
+          <t>Not sent - number is not on WhatsApp</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Queued for auto-send</t>
+          <t>Not sent - number is not on WhatsApp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Public phone +44 20 3417 3500; queued</t>
+          <t>Verified unavailable: +44 20 3417 3500 not on WhatsApp</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">

</xml_diff>

<commit_message>
Record contact channel priority rule
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,23 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>Active for every 10 AM run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Contact-channel priority</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Record every reliable public phone, WhatsApp number, email, contact form, or social-message channel with its source URL and use the available channel for outreach.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add email and phone outreach order
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -622,6 +622,23 @@
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Outreach order</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Attempt public email, then WhatsApp, then phone call or SMS when the connected adapter is available; record every result and never claim success without visible confirmation.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>

<commit_message>
Record No. 41 Coffee email delivery
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -861,7 +861,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Draft prepared for no41coffeekitchen@outlook.com</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Draft only</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Draft prepared; public email found</t>
+          <t>Sent to no41coffeekitchen@outlook.com</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">

</xml_diff>

<commit_message>
Send updated website screenshots by email
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1118,6 +1118,38 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>outreach/no-41-coffee.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>No. 41 Coffee</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sent - updated screenshots attached</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>no41coffeekitchen@outlook.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Updated ThemeWagon-based website preview and MultiMax introduction</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2 JPG attachments; Gmail message 1a159bd7d3b14d3f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record live GitHub Pages outreach
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sites/no-41-coffee/index.html</t>
+          <t>https://amalraj020-a11y.github.io/10-am-office-work/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Queued in current 10 AM run</t>
+          <t>GitHub Pages workflow success</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Sent with live link + screenshots</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1150,6 +1150,38 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>2 JPG attachments; Gmail message 1a159bd7d3b14d3f</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>No. 41 Coffee</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sent - deployed GitHub Pages link + screenshots</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>no41coffeekitchen@outlook.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Live preview: https://amalraj020-a11y.github.io/10-am-office-work/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2 JPG attachments; Gmail message 1a159d0b2852c7db</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add validated contact and GitHub Pages delivery rules
</commit_message>
<xml_diff>
--- a/work/10-am-office-work-tracker.xlsx
+++ b/work/10-am-office-work-tracker.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -639,6 +639,57 @@
         </is>
       </c>
       <c r="C10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Contact validation before build</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Verify discovered phone/WhatsApp usability and email validity through the connected adapters before starting website creation.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Approved template selection</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Choose and record a polished free template from the approved sources, especially ThemeWagon free catalog, including URL, repository, and license note.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Deployment and delivery sequence</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Deploy to GitHub Pages, verify the live URL, capture current screenshots, then send the live link and screenshots by email and WhatsApp when available; record every result.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>